<commit_message>
Botão de gerar certificado com pasta de destino
</commit_message>
<xml_diff>
--- a/historico/historico.xlsx
+++ b/historico/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -943,6 +943,21 @@
         <v>28</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Palestra Rock In Rio (respostas).xlsx</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:53</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>